<commit_message>
Add information and environment primitives
</commit_message>
<xml_diff>
--- a/benchmarking/system_benchmark_primitives.xlsx
+++ b/benchmarking/system_benchmark_primitives.xlsx
@@ -6,7 +6,8 @@
   </bookViews>
   <sheets>
     <sheet name="Primitive Values" sheetId="1" r:id="rId1"/>
-    <sheet name="Legend" sheetId="2" r:id="rId2"/>
+    <sheet name="Coverage Statistics" sheetId="2" r:id="rId2"/>
+    <sheet name="Legend" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
 </workbook>
@@ -95,7 +96,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -107,6 +108,9 @@
     <col min="7" max="7" width="58" customWidth="1"/>
     <col min="8" max="8" width="58" customWidth="1"/>
     <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="58" customWidth="1"/>
+    <col min="11" max="11" width="58" customWidth="1"/>
+    <col min="12" max="12" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -155,8 +159,23 @@
           <t xml:space="preserve">Motion Regime</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="48" customHeight="1">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observability / Information Gain</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic Environment</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Irreversibility</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="66" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">box-and-blocks</t>
@@ -202,8 +221,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="3" ht="48" customHeight="1">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — no unknown object properties must be identified</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — the task outcome is readily reversible</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="66" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">peg-in-hole</t>
@@ -249,8 +283,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="48" customHeight="1">
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — geometry and tolerances are specified</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — insertion can be reversed without material alteration</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="66" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">pick-up-flat-object</t>
@@ -296,8 +345,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="48" customHeight="1">
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — object and support properties are specified</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — lifting does not permanently alter the object</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="66" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">tie-a-knot</t>
@@ -343,8 +407,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="6" ht="48" customHeight="1">
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — rope configuration and tension must be inferred</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — material properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — the knot can be untied without material alteration</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="66" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">twist-lid-on-jar</t>
@@ -390,8 +469,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="48" customHeight="1">
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — thread engagement and seating must be detected</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — the lid can be unscrewed without material alteration</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="66" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">thread-screw-with-screwdriver</t>
@@ -437,8 +531,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="8" ht="48" customHeight="1">
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — engagement, cam-out, and seating must be detected</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — the screw can be removed without material alteration</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="66" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">cut-pattern-with-scissors</t>
@@ -484,8 +593,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — cut progress and paper state must be monitored</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — cutting changes the paper's connectivity</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High — cutting cannot be undone without repair or replacement</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="66" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">fasten-unfasten-button</t>
@@ -531,8 +655,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — buttonhole engagement and passage must be detected</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — material properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — fastening can be reversed without material alteration</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="66" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">in-hand-object-reorientation</t>
@@ -578,8 +717,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="48" customHeight="1">
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — object pose and slip must be estimated</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — reorientation does not permanently alter the object</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="66" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">spin-a-top</t>
@@ -625,8 +779,23 @@
           <t xml:space="preserve">Dynamic</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="48" customHeight="1">
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — no unknown object properties must be identified</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — spinning does not permanently alter the object</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="66" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">use-chopsticks</t>
@@ -672,8 +841,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="13" ht="48" customHeight="1">
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — capture and slip must be detected</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — transfers do not permanently alter the objects</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="66" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">extract-object-from-opaque-bag</t>
@@ -719,8 +903,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="14" ht="48" customHeight="1">
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High — active tactile exploration must identify the target</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — retrieval does not permanently alter the objects</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="66" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">bundle-socks</t>
@@ -766,8 +965,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="15" ht="48" customHeight="1">
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — garment shape and tension must be inferred</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — material properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — the socks can be unbundled without material alteration</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="66" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">zip-unzip-zipper</t>
@@ -813,8 +1027,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="48" customHeight="1">
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — slider engagement and fabric tension must be detected</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — material properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — closing is reversed within the task</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="66" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">paper-folding</t>
@@ -860,8 +1089,23 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="48" customHeight="1">
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — alignment, deformation, and crease state must be monitored</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — creasing changes local rest shape and stiffness</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — unfolding leaves a persistent crease</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="66" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">bundle-dowels-with-rubber-band</t>
@@ -907,9 +1151,24 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate — bundle geometry and band tension must be inferred</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — material properties remain effectively constant</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low — the bundle can be disassembled without material alteration</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I17"/>
+  <autoFilter ref="A1:L17"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -917,12 +1176,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="32" customWidth="1"/>
+    <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
-    <col min="3" max="3" width="100" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="90" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="7" width="82" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -938,11 +1201,1175 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Task Count</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Percent of Tasks</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tasks</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Category Breadth</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coverage Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="90" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manipulation</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Direct</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">81.3%</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Fasten Button, In-Hand Reorienting, Spin a Top, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2/2 categories (100.0%)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Both direct and indirect manipulation are represented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Manipulation</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Indirect</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18.8%</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use Screwdriver, Use Scissors, Use Chopsticks</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rigidity</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">8</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">50.0%</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Twist Lid on Jar, Use Screwdriver, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4/4 categories (100.0%)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All defined rigidity and environment categories are represented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rigidity</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Deformable manipulanda / rigid environment</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">18.8%</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tie a Knot, Bundle Socks, Paper Folding</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rigidity</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25.0%</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use Scissors, Fasten Button, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rigidity</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rigid manipulandum / environment not engaged</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3%</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">In-Hand Reorienting</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Relative Size</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smaller than the hand</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25.0%</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Pick Up Flat Object, Fasten Button, Spin a Top</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4/4 categories (100.0%)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">All defined relative-size categories are represented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Relative Size</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Comparable to the hand</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31.3%</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peg-in-Hole, Twist Lid on Jar, In-Hand Reorienting, Blindly Retrieve an Object from Cover, Bundle Socks</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Relative Size</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Larger than the hand</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3%</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper Folding</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Relative Size</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Mixed relative to the hand</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">37.5%</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tie a Knot, Use Screwdriver, Use Scissors, Use Chopsticks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controlled Degrees of Freedom</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31.3%</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Twist Lid on Jar, Spin a Top</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3/3 categories (100.0%)</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low, moderate, and high controlled-DoF tasks are represented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controlled Degrees of Freedom</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25.0%</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use Screwdriver, Fasten Button, Blindly Retrieve an Object from Cover, Zip a Zipper</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="90" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Controlled Degrees of Freedom</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">43.8%</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tie a Knot, Use Scissors, In-Hand Reorienting, Use Chopsticks, Bundle Socks, Paper Folding, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="90" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Constraint Complexity</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12.5%</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Spin a Top</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3/3 categories (100.0%)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low, moderate, and high constraint complexity are represented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="90" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Constraint Complexity</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31.3%</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use Scissors, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Paper Folding</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Constraint Complexity</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">56.3%</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Constraint Change</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.0%</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2/3 categories (66.7%)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coverage gap: no task has low constraint change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Constraint Change</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">37.5%</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Pick Up Flat Object, In-Hand Reorienting, Spin a Top, Use Chopsticks, Paper Folding</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Constraint Change</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">62.5%</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peg-in-Hole, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Motion Regime</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Quasistatic</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">15</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">93.8%</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2/2 categories (100.0%)</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic behavior is represented by only one task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Motion Regime</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3%</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Spin a Top</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observability / Information Gain</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">25.0%</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Spin a Top</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3/3 categories (100.0%)</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High information gain is represented by only one task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observability / Information Gain</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">68.8%</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Use Chopsticks, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="90" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observability / Information Gain</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3%</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blindly Retrieve an Object from Cover</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="90" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic Environment</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">87.5%</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2/3 categories (66.7%)</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coverage gap: no task has continuously changing object properties at the high level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="90" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic Environment</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12.5%</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use Scissors, Paper Folding</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic Environment</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.0%</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Irreversibility</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">87.5%</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3/3 categories (100.0%)</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate and high irreversibility are each represented by only one task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Irreversibility</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3%</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper Folding</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Irreversibility</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3%</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use Scissors</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G31"/>
+  <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C31"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="36" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+    <col min="3" max="3" width="105" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Primitive</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Definition</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1">
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Manipulation</t>
@@ -959,7 +2386,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Manipulation</t>
@@ -976,7 +2403,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="48" customHeight="1">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigidity</t>
@@ -993,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="48" customHeight="1">
+    <row r="5" ht="58" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigidity</t>
@@ -1010,7 +2437,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="48" customHeight="1">
+    <row r="6" ht="58" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigidity</t>
@@ -1027,7 +2454,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="48" customHeight="1">
+    <row r="7" ht="58" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigidity</t>
@@ -1044,7 +2471,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
+    <row r="8" ht="58" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Relative Size</t>
@@ -1061,7 +2488,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
+    <row r="9" ht="58" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Relative Size</t>
@@ -1078,7 +2505,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="48" customHeight="1">
+    <row r="10" ht="58" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Relative Size</t>
@@ -1095,7 +2522,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1">
+    <row r="11" ht="58" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Relative Size</t>
@@ -1112,7 +2539,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="48" customHeight="1">
+    <row r="12" ht="58" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Controlled Degrees of Freedom</t>
@@ -1129,7 +2556,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="48" customHeight="1">
+    <row r="13" ht="58" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Controlled Degrees of Freedom</t>
@@ -1146,7 +2573,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="48" customHeight="1">
+    <row r="14" ht="58" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Controlled Degrees of Freedom</t>
@@ -1163,7 +2590,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="48" customHeight="1">
+    <row r="15" ht="58" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Constraint Complexity</t>
@@ -1180,7 +2607,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
+    <row r="16" ht="58" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Constraint Complexity</t>
@@ -1197,7 +2624,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="48" customHeight="1">
+    <row r="17" ht="58" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Constraint Complexity</t>
@@ -1214,7 +2641,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="48" customHeight="1">
+    <row r="18" ht="58" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Constraint Change</t>
@@ -1222,68 +2649,238 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The active contact topology remains effectively constant throughout the task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="58" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Constraint Change</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Moderate</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">The task has a limited set of contact-mode transitions or repeats the same grasp, transport, and release cycle.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Constraint Change</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">The task has progressive or qualitatively different contact modes, self-contact, assembly, cutting, threading, wrapping, or active exploration.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21" ht="58" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Motion Regime</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Success does not require deliberate exploitation of momentum or other dynamic effects.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="48" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="22" ht="58" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Motion Regime</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Dynamic</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Success depends on deliberately generating or exploiting object dynamics.</t>
         </is>
       </c>
     </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observability / Information Gain</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Success does not require identifying unknown object properties or interaction states.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="58" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observability / Information Gain</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feedback must infer task-relevant contact, configuration, tension, slip, or engagement state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observability / Information Gain</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Active exploration and object identification are central to successful completion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="58" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic Environment</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The manipulanda retain effectively constant physical properties during the task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="58" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic Environment</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A localized or discrete operation persistently changes an object property, rest shape, or connectivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="58" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic Environment</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Continuously evolving object properties, such as changing damping, stiffness, curing, or jamming, are central to control.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="58" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Irreversibility</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The task outcome can be reversed without permanently altering or replacing material.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="58" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Irreversibility</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The operation can be functionally reversed, but a persistent residual material change remains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="58" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Irreversibility</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The original task state cannot be restored without repair or replacement.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C21"/>
+  <autoFilter ref="A1:C31"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Organize system benchmarks by task category
</commit_message>
<xml_diff>
--- a/benchmarking/system_benchmark_primitives.xlsx
+++ b/benchmarking/system_benchmark_primitives.xlsx
@@ -96,21 +96,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="50" customWidth="1"/>
-    <col min="7" max="7" width="58" customWidth="1"/>
+    <col min="3" max="3" width="42" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="28" customWidth="1"/>
+    <col min="7" max="7" width="50" customWidth="1"/>
     <col min="8" max="8" width="58" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
-    <col min="10" max="10" width="58" customWidth="1"/>
+    <col min="9" max="9" width="58" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
     <col min="11" max="11" width="58" customWidth="1"/>
     <col min="12" max="12" width="58" customWidth="1"/>
+    <col min="13" max="13" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -126,50 +127,55 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Task Category</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">Manipulation</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigidity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Relative Size</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Controlled Degrees of Freedom</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Constraint Complexity</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Constraint Change</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Motion Regime</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Observability / Information Gain</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Dynamic Environment</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Irreversibility</t>
         </is>
@@ -188,50 +194,55 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Object Transport and Retrieval</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Smaller than the hand</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — one rigid block at a time</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — repeated grasp, transport, and release</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — no unknown object properties must be identified</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — object properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — the task outcome is readily reversible</t>
         </is>
@@ -250,50 +261,55 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Assembly and Fastening</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Comparable to the hand</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — one rigid peg at a time</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — tight position and angle tolerances</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — free motion to constrained insertion</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — geometry and tolerances are specified</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — object properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — insertion can be reversed without material alteration</t>
         </is>
@@ -312,50 +328,55 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Object Transport and Retrieval</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Smaller than the hand</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — one rigid object</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — support severely restricts grasp contacts and approaches</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — table contact to hand support</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — object and support properties are specified</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — object properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — lifting does not permanently alter the object</t>
         </is>
@@ -374,50 +395,55 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Material Shaping and Reconfiguration</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Deformable manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed relative to the hand</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — continuously deformable rope</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — contact and topological constraints</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — evolving contacts and topology</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — rope configuration and tension must be inferred</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — material properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — the knot can be untied without material alteration</t>
         </is>
@@ -436,50 +462,55 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Assembly and Fastening</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Comparable to the hand</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — one movable rigid lid</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — threaded alignment and torque</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — free motion to thread engagement</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — thread engagement and seating must be detected</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — object properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — the lid can be unscrewed without material alteration</t>
         </is>
@@ -498,50 +529,55 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Assembly and Fastening</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Indirect — tool use</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed relative to the hand</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — tool pose plus constrained screw motion</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — alignment, axial force, and torque</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — transport, engagement, and tightening</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="J7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — engagement, cam-out, and seating must be detected</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — object properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — the screw can be removed without material alteration</t>
         </is>
@@ -560,50 +596,55 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Opening, Separation, and Disassembly</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Indirect — articulated tool</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed relative to the hand</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — tool articulation and sheet control</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — path following, blade contact, and material support</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — repeated blade-material contact</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — cut progress and paper state must be monitored</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — cutting changes the paper's connectivity</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — cutting cannot be undone without repair or replacement</t>
         </is>
@@ -622,50 +663,55 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Assembly and Fastening</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Smaller than the hand</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — object pose and localized fabric deformation</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — tight geometry and force coordination</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — contact, partial insertion, and passage</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="J9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — buttonhole engagement and passage must be detected</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="L9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — material properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L9" s="3" t="inlineStr">
+      <c r="M9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — fastening can be reversed without material alteration</t>
         </is>
@@ -684,50 +730,55 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Material Shaping and Reconfiguration</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigid manipulandum / environment not engaged</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Comparable to the hand</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — object pose and multiple finger joints</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — simultaneous contacts and grasp forces</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — contacts shift without release</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — object pose and slip must be estimated</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — object properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — reorientation does not permanently alter the object</t>
         </is>
@@ -746,50 +797,55 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Dynamic Manipulation</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Smaller than the hand</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — one rigid object</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — few simultaneous environmental constraints</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — grasp, release, and table contact</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="J11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Dynamic</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — no unknown object properties must be identified</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — object properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — spinning does not permanently alter the object</t>
         </is>
@@ -808,50 +864,55 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Object Transport and Retrieval</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Indirect — two tools</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed relative to the hand</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — two tools and object pose</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — bilateral contact and force regulation</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — repeated acquisition and release cycles</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — capture and slip must be detected</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — object properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — transfers do not permanently alter the objects</t>
         </is>
@@ -870,50 +931,55 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Object Transport and Retrieval</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Comparable to the hand</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — target pose amid movable distractors</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — clutter and confinement</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — exploratory contacts form and break</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="J13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — active tactile exploration must identify the target</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="L13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — object properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L13" s="3" t="inlineStr">
+      <c r="M13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — retrieval does not permanently alter the objects</t>
         </is>
@@ -932,50 +998,55 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Material Shaping and Reconfiguration</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Deformable manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Comparable to the hand</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — two continuously deformable objects</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — compliant alignment, rolling, and tucking</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="I14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — repeated folding, stretching, and contact</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — garment shape and tension must be inferred</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — material properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — the socks can be unbundled without material alteration</t>
         </is>
@@ -994,50 +1065,55 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Assembly and Fastening</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed relative to the hand</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — guided slider and constrained fabric deformation</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — alignment, tension, and guided motion</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — engagement and disengagement</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="J15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — slider engagement and fabric tension must be detected</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="L15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — material properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — closing is reversed within the task</t>
         </is>
@@ -1056,50 +1132,55 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Material Shaping and Reconfiguration</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Deformable manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Larger than the hand</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High — distributed sheet deformation</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — edge alignment and crease tolerance</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — support, folding, self-contact, and release</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — alignment, deformation, and crease state must be monitored</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — creasing changes local rest shape and stiffness</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — unfolding leaves a persistent crease</t>
         </is>
@@ -1118,57 +1199,62 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Assembly and Fastening</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mixed relative to the hand</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — seven objects and an elastic fastener</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — alignment, compression, and wrapping</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">High — gathering, stretching, and securing</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Moderate — bundle geometry and band tension must be inferred</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="L17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — material properties remain effectively constant</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Low — the bundle can be disassembled without material alteration</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L17"/>
+  <autoFilter ref="A1:M17"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
@@ -1176,7 +1262,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -1228,64 +1314,64 @@
     <row r="2" ht="90" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manipulation</t>
+          <t xml:space="preserve">Task Category</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t xml:space="preserve">Object Transport and Retrieval</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">13</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">81.3%</t>
+          <t xml:space="preserve">25.0%</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Fasten Button, In-Hand Reorienting, Spin a Top, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
+          <t xml:space="preserve">Box and Blocks, Pick Up Flat Object, Use Chopsticks, Blindly Retrieve an Object from Cover</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/2 categories (100.0%)</t>
+          <t xml:space="preserve">5/5 categories (100.0%)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Both direct and indirect manipulation are represented.</t>
+          <t xml:space="preserve">All defined task categories are represented.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="90" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manipulation</t>
+          <t xml:space="preserve">Task Category</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indirect</t>
+          <t xml:space="preserve">Assembly and Fastening</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.8%</t>
+          <t xml:space="preserve">37.5%</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Screwdriver, Use Scissors, Use Chopsticks</t>
+          <t xml:space="preserve">Peg-in-Hole, Twist Lid on Jar, Use Screwdriver, Fasten Button, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -1302,64 +1388,64 @@
     <row r="4" ht="90" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigidity</t>
+          <t xml:space="preserve">Task Category</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
+          <t xml:space="preserve">Material Shaping and Reconfiguration</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">50.0%</t>
+          <t xml:space="preserve">25.0%</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Twist Lid on Jar, Use Screwdriver, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover</t>
+          <t xml:space="preserve">Tie a Knot, In-Hand Reorienting, Bundle Socks, Paper Folding</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4/4 categories (100.0%)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">All defined rigidity and environment categories are represented.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigidity</t>
+          <t xml:space="preserve">Task Category</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deformable manipulanda / rigid environment</t>
+          <t xml:space="preserve">Opening, Separation, and Disassembly</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.8%</t>
+          <t xml:space="preserve">6.3%</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie a Knot, Bundle Socks, Paper Folding</t>
+          <t xml:space="preserve">Use Scissors</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1376,27 +1462,27 @@
     <row r="6" ht="90" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigidity</t>
+          <t xml:space="preserve">Task Category</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
+          <t xml:space="preserve">Dynamic Manipulation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25.0%</t>
+          <t xml:space="preserve">6.3%</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Scissors, Fasten Button, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t xml:space="preserve">Spin a Top</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1413,138 +1499,138 @@
     <row r="7" ht="90" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigidity</t>
+          <t xml:space="preserve">Manipulation</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulandum / environment not engaged</t>
+          <t xml:space="preserve">Direct</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">13</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t xml:space="preserve">81.3%</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">In-Hand Reorienting</t>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Fasten Button, In-Hand Reorienting, Spin a Top, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2/2 categories (100.0%)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Both direct and indirect manipulation are represented.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="90" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relative Size</t>
+          <t xml:space="preserve">Manipulation</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smaller than the hand</t>
+          <t xml:space="preserve">Indirect</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25.0%</t>
+          <t xml:space="preserve">18.8%</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Pick Up Flat Object, Fasten Button, Spin a Top</t>
+          <t xml:space="preserve">Use Screwdriver, Use Scissors, Use Chopsticks</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4/4 categories (100.0%)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">All defined relative-size categories are represented.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relative Size</t>
+          <t xml:space="preserve">Rigidity</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparable to the hand</t>
+          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">31.3%</t>
+          <t xml:space="preserve">50.0%</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peg-in-Hole, Twist Lid on Jar, In-Hand Reorienting, Blindly Retrieve an Object from Cover, Bundle Socks</t>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Twist Lid on Jar, Use Screwdriver, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">4/4 categories (100.0%)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">All defined rigidity and environment categories are represented.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relative Size</t>
+          <t xml:space="preserve">Rigidity</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Larger than the hand</t>
+          <t xml:space="preserve">Deformable manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t xml:space="preserve">18.8%</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paper Folding</t>
+          <t xml:space="preserve">Tie a Knot, Bundle Socks, Paper Folding</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1561,27 +1647,27 @@
     <row r="11" ht="90" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relative Size</t>
+          <t xml:space="preserve">Rigidity</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed relative to the hand</t>
+          <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">37.5%</t>
+          <t xml:space="preserve">25.0%</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie a Knot, Use Screwdriver, Use Scissors, Use Chopsticks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t xml:space="preserve">Use Scissors, Fasten Button, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1598,49 +1684,49 @@
     <row r="12" ht="90" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Controlled Degrees of Freedom</t>
+          <t xml:space="preserve">Rigidity</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low</t>
+          <t xml:space="preserve">Rigid manipulandum / environment not engaged</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">31.3%</t>
+          <t xml:space="preserve">6.3%</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Twist Lid on Jar, Spin a Top</t>
+          <t xml:space="preserve">In-Hand Reorienting</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3/3 categories (100.0%)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low, moderate, and high controlled-DoF tasks are represented.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Controlled Degrees of Freedom</t>
+          <t xml:space="preserve">Relative Size</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate</t>
+          <t xml:space="preserve">Smaller than the hand</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1655,44 +1741,44 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Screwdriver, Fasten Button, Blindly Retrieve an Object from Cover, Zip a Zipper</t>
+          <t xml:space="preserve">Box and Blocks, Pick Up Flat Object, Fasten Button, Spin a Top</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">4/4 categories (100.0%)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">All defined relative-size categories are represented.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="90" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Controlled Degrees of Freedom</t>
+          <t xml:space="preserve">Relative Size</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t xml:space="preserve">Comparable to the hand</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">43.8%</t>
+          <t xml:space="preserve">31.3%</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie a Knot, Use Scissors, In-Hand Reorienting, Use Chopsticks, Bundle Socks, Paper Folding, Bundle Dowels with a Rubber Band</t>
+          <t xml:space="preserve">Peg-in-Hole, Twist Lid on Jar, In-Hand Reorienting, Blindly Retrieve an Object from Cover, Bundle Socks</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1709,64 +1795,64 @@
     <row r="15" ht="90" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constraint Complexity</t>
+          <t xml:space="preserve">Relative Size</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low</t>
+          <t xml:space="preserve">Larger than the hand</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12.5%</t>
+          <t xml:space="preserve">6.3%</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Spin a Top</t>
+          <t xml:space="preserve">Paper Folding</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3/3 categories (100.0%)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low, moderate, and high constraint complexity are represented.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="16" ht="90" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constraint Complexity</t>
+          <t xml:space="preserve">Relative Size</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate</t>
+          <t xml:space="preserve">Mixed relative to the hand</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">31.3%</t>
+          <t xml:space="preserve">37.5%</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Scissors, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Paper Folding</t>
+          <t xml:space="preserve">Tie a Knot, Use Screwdriver, Use Scissors, Use Chopsticks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1783,101 +1869,101 @@
     <row r="17" ht="90" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constraint Complexity</t>
+          <t xml:space="preserve">Controlled Degrees of Freedom</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t xml:space="preserve">Low</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">56.3%</t>
+          <t xml:space="preserve">31.3%</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Twist Lid on Jar, Spin a Top</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3/3 categories (100.0%)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Low, moderate, and high controlled-DoF tasks are represented.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constraint Change</t>
+          <t xml:space="preserve">Controlled Degrees of Freedom</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low</t>
+          <t xml:space="preserve">Moderate</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0%</t>
+          <t xml:space="preserve">25.0%</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Use Screwdriver, Fasten Button, Blindly Retrieve an Object from Cover, Zip a Zipper</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/3 categories (66.7%)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coverage gap: no task has low constraint change.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="19" ht="90" customHeight="1">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constraint Change</t>
+          <t xml:space="preserve">Controlled Degrees of Freedom</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate</t>
+          <t xml:space="preserve">High</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">37.5%</t>
+          <t xml:space="preserve">43.8%</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Pick Up Flat Object, In-Hand Reorienting, Spin a Top, Use Chopsticks, Paper Folding</t>
+          <t xml:space="preserve">Tie a Knot, Use Scissors, In-Hand Reorienting, Use Chopsticks, Bundle Socks, Paper Folding, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1894,101 +1980,101 @@
     <row r="20" ht="90" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Constraint Change</t>
+          <t xml:space="preserve">Constraint Complexity</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t xml:space="preserve">Low</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">62.5%</t>
+          <t xml:space="preserve">12.5%</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peg-in-Hole, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t xml:space="preserve">Box and Blocks, Spin a Top</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3/3 categories (100.0%)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Low, moderate, and high constraint complexity are represented.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="90" customHeight="1">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Motion Regime</t>
+          <t xml:space="preserve">Constraint Complexity</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t xml:space="preserve">Moderate</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t xml:space="preserve">5</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">93.8%</t>
+          <t xml:space="preserve">31.3%</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
+          <t xml:space="preserve">Use Scissors, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Paper Folding</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/2 categories (100.0%)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dynamic behavior is represented by only one task.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="22" ht="90" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Motion Regime</t>
+          <t xml:space="preserve">Constraint Complexity</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dynamic</t>
+          <t xml:space="preserve">High</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t xml:space="preserve">56.3%</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spin a Top</t>
+          <t xml:space="preserve">Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -2005,7 +2091,7 @@
     <row r="23" ht="90" customHeight="1">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Observability / Information Gain</t>
+          <t xml:space="preserve">Constraint Change</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -2015,34 +2101,34 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">25.0%</t>
+          <t xml:space="preserve">0.0%</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Spin a Top</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3/3 categories (100.0%)</t>
+          <t xml:space="preserve">2/3 categories (66.7%)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High information gain is represented by only one task.</t>
+          <t xml:space="preserve">Coverage gap: no task has low constraint change.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="90" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Observability / Information Gain</t>
+          <t xml:space="preserve">Constraint Change</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -2052,17 +2138,17 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">11</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">68.8%</t>
+          <t xml:space="preserve">37.5%</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Use Chopsticks, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
+          <t xml:space="preserve">Box and Blocks, Pick Up Flat Object, In-Hand Reorienting, Spin a Top, Use Chopsticks, Paper Folding</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2079,7 +2165,7 @@
     <row r="25" ht="90" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Observability / Information Gain</t>
+          <t xml:space="preserve">Constraint Change</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -2089,17 +2175,17 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">1</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t xml:space="preserve">62.5%</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blindly Retrieve an Object from Cover</t>
+          <t xml:space="preserve">Peg-in-Hole, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -2116,64 +2202,64 @@
     <row r="26" ht="90" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dynamic Environment</t>
+          <t xml:space="preserve">Motion Regime</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low</t>
+          <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">14</t>
+          <t xml:space="preserve">15</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">87.5%</t>
+          <t xml:space="preserve">93.8%</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/3 categories (66.7%)</t>
+          <t xml:space="preserve">2/2 categories (100.0%)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coverage gap: no task has continuously changing object properties at the high level.</t>
+          <t xml:space="preserve">Dynamic behavior is represented by only one task.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="90" customHeight="1">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dynamic Environment</t>
+          <t xml:space="preserve">Motion Regime</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate</t>
+          <t xml:space="preserve">Dynamic</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">12.5%</t>
+          <t xml:space="preserve">6.3%</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Scissors, Paper Folding</t>
+          <t xml:space="preserve">Spin a Top</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -2190,86 +2276,86 @@
     <row r="28" ht="90" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dynamic Environment</t>
+          <t xml:space="preserve">Observability / Information Gain</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High</t>
+          <t xml:space="preserve">Low</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0%</t>
+          <t xml:space="preserve">25.0%</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Spin a Top</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">3/3 categories (100.0%)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">High information gain is represented by only one task.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="90" customHeight="1">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Irreversibility</t>
+          <t xml:space="preserve">Observability / Information Gain</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low</t>
+          <t xml:space="preserve">Moderate</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">14</t>
+          <t xml:space="preserve">11</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">87.5%</t>
+          <t xml:space="preserve">68.8%</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t xml:space="preserve">Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Use Chopsticks, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3/3 categories (100.0%)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate and high irreversibility are each represented by only one task.</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="30" ht="90" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Irreversibility</t>
+          <t xml:space="preserve">Observability / Information Gain</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate</t>
+          <t xml:space="preserve">High</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2284,7 +2370,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paper Folding</t>
+          <t xml:space="preserve">Blindly Retrieve an Object from Cover</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2301,42 +2387,227 @@
     <row r="31" ht="90" customHeight="1">
       <c r="A31" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">Dynamic Environment</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">87.5%</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2/3 categories (66.7%)</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Coverage gap: no task has continuously changing object properties at the high level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic Environment</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">12.5%</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use Scissors, Paper Folding</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dynamic Environment</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.0%</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Irreversibility</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">14</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">87.5%</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3/3 categories (100.0%)</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate and high irreversibility are each represented by only one task.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="90" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Irreversibility</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Moderate</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6.3%</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Paper Folding</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Irreversibility</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">High</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">6.3%</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Use Scissors</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G31"/>
+  <autoFilter ref="A1:G36"/>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Align primitive descriptions with benchmark task requirements
</commit_message>
<xml_diff>
--- a/benchmarking/system_benchmark_primitives.xlsx
+++ b/benchmarking/system_benchmark_primitives.xlsx
@@ -425,7 +425,7 @@
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — evolving contacts and topology</t>
+          <t xml:space="preserve">High — evolving self-contacts and threading constraints</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — transport, engagement, and tightening</t>
+          <t xml:space="preserve">High — tool acquisition, engagement, rotation, and disengagement</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — repeated folding, stretching, and contact</t>
+          <t xml:space="preserve">High — rolling, cuff stretching, and tucking</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -2653,7 +2653,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The hand contacts and manipulates the task object directly.</t>
+          <t xml:space="preserve">The hand acts directly on the relevant object or mechanism.</t>
         </is>
       </c>
     </row>
@@ -2670,7 +2670,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The hand acts on the task object through an intermediate tool.</t>
+          <t xml:space="preserve">One or more tools transmit the hand’s action to the object. Other direct contacts, such as supporting paper during cutting, may still occur.</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">All manipulated objects and the active environment are rigid.</t>
+          <t xml:space="preserve">The handled objects and tools are effectively rigid, and the task uses a rigid support or fixture.</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The manipulated objects deform while the active environment is rigid.</t>
+          <t xml:space="preserve">The handled objects deform, and the task uses a rigid support or fixture during setup, manipulation, or release.</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The task combines rigid and deformable manipulated objects in a rigid environment.</t>
+          <t xml:space="preserve">The task coordinates rigid components or tools with deformable material, using a rigid support or fixture.</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A rigid object is manipulated without contacting or using the environment.</t>
+          <t xml:space="preserve">The rigid object stays within the hand, and environmental contact is excluded throughout the trial.</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The relevant manipulated object is smaller than the hand.</t>
+          <t xml:space="preserve">The primary handled object or local component is smaller than the hand.</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The relevant manipulated object is approximately hand-scale.</t>
+          <t xml:space="preserve">The relevant object’s overall extent is approximately the size of the hand.</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The relevant manipulated object is larger than the hand.</t>
+          <t xml:space="preserve">The relevant object extends beyond the hand over the area being manipulated.</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Different manipulanda, or different dimensions of one manipulandum, span multiple size categories.</t>
+          <t xml:space="preserve">Relevant tools and objects span different sizes, or a slender object is longer than the hand while its graspable cross-section is smaller.</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">One rigid body is intentionally controlled at a time.</t>
+          <t xml:space="preserve">One rigid object’s pose or motion is controlled through a simple grasp, with no required sustained reconfiguration of finger contacts or coordination of additional movable components.</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2840,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The task controls coupled rigid bodies or localized or fixture-constrained deformation.</t>
+          <t xml:space="preserve">Limited additional coordination is required for guided mechanism motion, localized deformation, or movable distractors during confined exploration.</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The task controls several bodies, distributed deformation, or changing multi-contact coordination.</t>
+          <t xml:space="preserve">The task requires coordinating several independently controlled objects or tool elements, distributed deformation, or sustained independent motion of finger contacts and object pose.</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Few loose constraints are active, without tight mating or substantial force regulation.</t>
+          <t xml:space="preserve">Few physical constraints are active together, with broad freedom to choose contacts and motion. Speed or precise release timing can still be demanding.</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The task includes restricted access, path or pose tolerances, clutter, or limited force regulation.</t>
+          <t xml:space="preserve">The task requires path or edge alignment, managing clutter and confinement, compliant positioning, or simple opposing-contact force regulation, while leaving multiple feasible ways to satisfy those requirements.</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The task includes tight mating, severe access restriction, multiple simultaneous contacts, topology, or strong force and impedance requirements.</t>
+          <t xml:space="preserve">Tight mating geometry, severely restricted grasp access, knot topology, or interdependent alignment and contact-force requirements sharply restrict feasible motions or grasps.</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The active contact topology remains effectively constant throughout the task.</t>
+          <t xml:space="preserve">The contact arrangement and motion restrictions remain effectively constant throughout the task.</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The task has a limited set of contact-mode transitions or repeats the same grasp, transport, and release cycle.</t>
+          <t xml:space="preserve">Contacts follow a limited sequence, shift within a continuously controlled grasp, or repeat the same acquisition-and-release cycle. A single fold with support, self-contact, and release also falls here.</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The task has progressive or qualitatively different contact modes, self-contact, assembly, cutting, threading, wrapping, or active exploration.</t>
+          <t xml:space="preserve">Contacts progressively impose new motion restrictions, engage or disengage along an interface, or repeatedly reorganize during cutting, exploration, knotting, rolling and tucking, or wrapping.</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Success does not require deliberate exploitation of momentum or other dynamic effects.</t>
+          <t xml:space="preserve">Success can be achieved through controlled positioning and contact forces without deliberately exploiting momentum or free motion. A time limit alone does not change this rating.</t>
         </is>
       </c>
     </row>
@@ -2993,7 +2993,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Success depends on deliberately generating or exploiting object dynamics.</t>
+          <t xml:space="preserve">Success deliberately uses momentum or inertial effects. For Spin a Top, the imparted angular velocity and release conditions determine whether the top continues spinning upright.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Shorten primitive value descriptions and remove examples
</commit_message>
<xml_diff>
--- a/benchmarking/system_benchmark_primitives.xlsx
+++ b/benchmarking/system_benchmark_primitives.xlsx
@@ -2653,7 +2653,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The hand acts directly on the relevant object or mechanism.</t>
+          <t xml:space="preserve">The hand acts directly on the task object.</t>
         </is>
       </c>
     </row>
@@ -2670,7 +2670,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">One or more tools transmit the hand’s action to the object. Other direct contacts, such as supporting paper during cutting, may still occur.</t>
+          <t xml:space="preserve">Tools transmit the hand’s action to the task object.</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2687,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The handled objects and tools are effectively rigid, and the task uses a rigid support or fixture.</t>
+          <t xml:space="preserve">Rigid objects and tools interact with rigid supports or fixtures.</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2704,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The handled objects deform, and the task uses a rigid support or fixture during setup, manipulation, or release.</t>
+          <t xml:space="preserve">Deformable objects are handled using rigid supports or fixtures.</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The task coordinates rigid components or tools with deformable material, using a rigid support or fixture.</t>
+          <t xml:space="preserve">Rigid and deformable components are handled together in a rigid environment.</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The rigid object stays within the hand, and environmental contact is excluded throughout the trial.</t>
+          <t xml:space="preserve">A rigid object is manipulated within the hand without environmental contact.</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The primary handled object or local component is smaller than the hand.</t>
+          <t xml:space="preserve">The main handled object or component is smaller than the hand.</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2772,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The relevant object’s overall extent is approximately the size of the hand.</t>
+          <t xml:space="preserve">The handled object is approximately the size of the hand.</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2789,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The relevant object extends beyond the hand over the area being manipulated.</t>
+          <t xml:space="preserve">The handled object extends beyond the hand’s size.</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relevant tools and objects span different sizes, or a slender object is longer than the hand while its graspable cross-section is smaller.</t>
+          <t xml:space="preserve">Handled components or relevant dimensions span multiple size categories.</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">One rigid object’s pose or motion is controlled through a simple grasp, with no required sustained reconfiguration of finger contacts or coordination of additional movable components.</t>
+          <t xml:space="preserve">One rigid object is controlled with a simple grasp and minimal contact reconfiguration.</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2840,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Limited additional coordination is required for guided mechanism motion, localized deformation, or movable distractors during confined exploration.</t>
+          <t xml:space="preserve">Guided mechanisms, localized deformation, or movable distractors require limited additional coordination.</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The task requires coordinating several independently controlled objects or tool elements, distributed deformation, or sustained independent motion of finger contacts and object pose.</t>
+          <t xml:space="preserve">Multiple objects, distributed deformation, or independent finger-contact motion require substantial coordination.</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2874,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Few physical constraints are active together, with broad freedom to choose contacts and motion. Speed or precise release timing can still be demanding.</t>
+          <t xml:space="preserve">Few simultaneous constraints leave broad freedom in grasp and motion.</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The task requires path or edge alignment, managing clutter and confinement, compliant positioning, or simple opposing-contact force regulation, while leaving multiple feasible ways to satisfy those requirements.</t>
+          <t xml:space="preserve">Alignment, confinement, or contact-force requirements allow several feasible manipulation strategies.</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tight mating geometry, severely restricted grasp access, knot topology, or interdependent alignment and contact-force requirements sharply restrict feasible motions or grasps.</t>
+          <t xml:space="preserve">Tight geometry, restricted access, topology, or coupled force requirements severely limit feasible grasps and motions.</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2925,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The contact arrangement and motion restrictions remain effectively constant throughout the task.</t>
+          <t xml:space="preserve">Contacts and motion restrictions remain effectively constant.</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contacts follow a limited sequence, shift within a continuously controlled grasp, or repeat the same acquisition-and-release cycle. A single fold with support, self-contact, and release also falls here.</t>
+          <t xml:space="preserve">Contacts follow a limited sequence, shift within a grasp, or repeat the same handling cycle.</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contacts progressively impose new motion restrictions, engage or disengage along an interface, or repeatedly reorganize during cutting, exploration, knotting, rolling and tucking, or wrapping.</t>
+          <t xml:space="preserve">Contact modes progressively restrict motion or repeatedly reorganize across interfaces or deformable objects.</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2976,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Success can be achieved through controlled positioning and contact forces without deliberately exploiting momentum or free motion. A time limit alone does not change this rating.</t>
+          <t xml:space="preserve">Controlled positioning and contact forces suffice; exploiting momentum is unnecessary.</t>
         </is>
       </c>
     </row>
@@ -2993,7 +2993,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Success deliberately uses momentum or inertial effects. For Spin a Top, the imparted angular velocity and release conditions determine whether the top continues spinning upright.</t>
+          <t xml:space="preserve">Success requires deliberately generating or exploiting momentum and inertial effects.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify benchmark instructions, primitives, and configuration images
</commit_message>
<xml_diff>
--- a/benchmarking/system_benchmark_primitives.xlsx
+++ b/benchmarking/system_benchmark_primitives.xlsx
@@ -199,52 +199,52 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
+          <t>Rigid manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smaller than the hand</t>
+          <t>Smaller than the hand</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — one rigid block at a time</t>
+          <t>Low — one rigid block at a time</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — repeated grasp, transport, and release</t>
+          <t>Moderate — repeated grasp, transport, and release</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — no unknown object properties must be identified</t>
+          <t>Low — no unknown object properties must be identified</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+          <t>Low — object properties remain effectively constant</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — the task outcome is readily reversible</t>
+          <t>Low — the task outcome is readily reversible</t>
         </is>
       </c>
     </row>
@@ -266,52 +266,52 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
+          <t>Rigid manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparable to the hand</t>
+          <t>Comparable to the hand</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — one rigid peg at a time</t>
+          <t>Low — one rigid peg at a time</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — tight position and angle tolerances</t>
+          <t>High — tight position and angle tolerances</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — free motion to constrained insertion</t>
+          <t>High — free motion to constrained insertion</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — geometry and tolerances are specified</t>
+          <t>Low — geometry and tolerances are specified</t>
         </is>
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+          <t>Low — object properties remain effectively constant</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — insertion can be reversed without material alteration</t>
+          <t>Low — insertion can be reversed without material alteration</t>
         </is>
       </c>
     </row>
@@ -333,52 +333,52 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
+          <t>Rigid manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smaller than the hand</t>
+          <t>Smaller than the hand</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — one rigid object</t>
+          <t>Low — one rigid object</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — support severely restricts grasp contacts and approaches</t>
+          <t>High — support severely restricts grasp contacts and approaches</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — table contact to hand support</t>
+          <t>Moderate — table contact to hand support</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — object and support properties are specified</t>
+          <t>Low — object and support properties are specified</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+          <t>Low — object properties remain effectively constant</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — lifting does not permanently alter the object</t>
+          <t>Low — lifting does not permanently alter the object</t>
         </is>
       </c>
     </row>
@@ -400,52 +400,52 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deformable manipulanda / rigid environment</t>
+          <t>Deformable manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed relative to the hand</t>
+          <t>Mixed relative to the hand</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — continuously deformable rope</t>
+          <t>High — continuously deformable rope</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — contact and topological constraints</t>
+          <t>High — contact and topological constraints</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — evolving self-contacts and threading constraints</t>
+          <t>High — evolving self-contacts and threading constraints</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — rope configuration and tension must be inferred</t>
+          <t>Moderate — rope configuration and tension must be inferred</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — material properties remain effectively constant</t>
+          <t>Low — material properties remain effectively constant</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — the knot can be untied without material alteration</t>
+          <t>Low — the knot can be untied without material alteration</t>
         </is>
       </c>
     </row>
@@ -467,52 +467,52 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
+          <t>Rigid manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparable to the hand</t>
+          <t>Comparable to the hand</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — one movable rigid lid</t>
+          <t>Low — one movable rigid lid</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — threaded alignment and torque</t>
+          <t>High — threaded alignment and torque</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — free motion to thread engagement</t>
+          <t>High — free motion to thread engagement</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — thread engagement and seating must be detected</t>
+          <t>Moderate — thread engagement and seating must be detected</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+          <t>Low — object properties remain effectively constant</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — the lid can be unscrewed without material alteration</t>
+          <t>Low — the lid can be unscrewed without material alteration</t>
         </is>
       </c>
     </row>
@@ -534,52 +534,52 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indirect — tool use</t>
+          <t>Indirect — tool use</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
+          <t>Rigid manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed relative to the hand</t>
+          <t>Mixed relative to the hand</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — tool pose plus constrained screw motion</t>
+          <t>Moderate — tool pose plus constrained screw motion</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — alignment, axial force, and torque</t>
+          <t>High — alignment, axial force, and torque</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — tool acquisition, engagement, rotation, and disengagement</t>
+          <t>High — tool acquisition, engagement, rotation, and disengagement</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — engagement, cam-out, and seating must be detected</t>
+          <t>Moderate — engagement, cam-out, and seating must be detected</t>
         </is>
       </c>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+          <t>Low — object properties remain effectively constant</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — the screw can be removed without material alteration</t>
+          <t>Low — the screw can be removed without material alteration</t>
         </is>
       </c>
     </row>
@@ -601,52 +601,52 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indirect — articulated tool</t>
+          <t>Indirect — articulated tool</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
+          <t>Mixed manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed relative to the hand</t>
+          <t>Mixed relative to the hand</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — tool articulation and sheet control</t>
+          <t>High — tool articulation and sheet control</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — path following, blade contact, and material support</t>
+          <t>Moderate — path following, blade contact, and material support</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — repeated blade-material contact</t>
+          <t>High — repeated blade-material contact</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — cut progress and paper state must be monitored</t>
+          <t>Moderate — cut progress and paper state must be monitored</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — cutting changes the paper's connectivity</t>
+          <t>Moderate — cutting changes the paper's connectivity</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — cutting cannot be undone without repair or replacement</t>
+          <t>High — cutting cannot be undone without repair or replacement</t>
         </is>
       </c>
     </row>
@@ -668,52 +668,52 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
+          <t>Mixed manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smaller than the hand</t>
+          <t>Smaller than the hand</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — object pose and localized fabric deformation</t>
+          <t>Moderate — object pose and localized fabric deformation</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — tight geometry and force coordination</t>
+          <t>High — tight geometry and force coordination</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — contact, partial insertion, and passage</t>
+          <t>High — contact, partial insertion, and passage</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — buttonhole engagement and passage must be detected</t>
+          <t>Moderate — buttonhole engagement and passage must be detected</t>
         </is>
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — material properties remain effectively constant</t>
+          <t>Low — material properties remain effectively constant</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — fastening can be reversed without material alteration</t>
+          <t>Low — fastening can be reversed without material alteration</t>
         </is>
       </c>
     </row>
@@ -735,52 +735,52 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulandum / environment not engaged</t>
+          <t>Rigid manipulandum / environment not engaged</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparable to the hand</t>
+          <t>Comparable to the hand</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — object pose and multiple finger joints</t>
+          <t>Low — one rigid object</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — simultaneous contacts and grasp forces</t>
+          <t>High — simultaneous rolling, sliding, and sticking contacts</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — contacts shift without release</t>
+          <t>High — rolling, sliding, and sticking contact modes form and break</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — object pose and slip must be estimated</t>
+          <t>Moderate — object pose and slip must be estimated</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+          <t>Low — object properties remain effectively constant</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — reorientation does not permanently alter the object</t>
+          <t>Low — reorientation does not permanently alter the object</t>
         </is>
       </c>
     </row>
@@ -802,52 +802,52 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
+          <t>Rigid manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smaller than the hand</t>
+          <t>Smaller than the hand</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — one rigid object</t>
+          <t>Low — one rigid object</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — few simultaneous environmental constraints</t>
+          <t>Low — few simultaneous environmental constraints</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — grasp, release, and table contact</t>
+          <t>Moderate — grasp, release, and table contact</t>
         </is>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dynamic</t>
+          <t>Dynamic</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — no unknown object properties must be identified</t>
+          <t>Low — no unknown object properties must be identified</t>
         </is>
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+          <t>Low — object properties remain effectively constant</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — spinning does not permanently alter the object</t>
+          <t>Low — spinning does not permanently alter the object</t>
         </is>
       </c>
     </row>
@@ -869,52 +869,52 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Indirect — two tools</t>
+          <t>Indirect — two tools</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
+          <t>Rigid manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed relative to the hand</t>
+          <t>Mixed relative to the hand</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — two tools and object pose</t>
+          <t>High — two tools and object pose</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — bilateral contact and force regulation</t>
+          <t>Moderate — two-sided contact and force regulation</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — repeated acquisition and release cycles</t>
+          <t>Moderate — repeated acquisition and release cycles</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — capture and slip must be detected</t>
+          <t>Moderate — capture and slip must be detected</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+          <t>Low — object properties remain effectively constant</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — transfers do not permanently alter the objects</t>
+          <t>Low — transfers do not permanently alter the objects</t>
         </is>
       </c>
     </row>
@@ -936,52 +936,52 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
+          <t>Rigid manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparable to the hand</t>
+          <t>Comparable to the hand</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — target pose amid movable distractors</t>
+          <t>Moderate — target pose amid movable distractors</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — clutter and confinement</t>
+          <t>Moderate — clutter and confinement</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — exploratory contacts form and break</t>
+          <t>High — exploratory contacts form and break</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — active tactile exploration must identify the target</t>
+          <t>High — active tactile exploration must identify the target</t>
         </is>
       </c>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — object properties remain effectively constant</t>
+          <t>Low — object properties remain effectively constant</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — retrieval does not permanently alter the objects</t>
+          <t>Low — retrieval does not permanently alter the objects</t>
         </is>
       </c>
     </row>
@@ -1003,52 +1003,52 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deformable manipulanda / rigid environment</t>
+          <t>Deformable manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparable to the hand</t>
+          <t>Comparable to the hand</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — two continuously deformable objects</t>
+          <t>High — two continuously deformable objects</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — compliant alignment, rolling, and tucking</t>
+          <t>High — coupled rolling, tucking, and deformable self-contact constraints</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — rolling, cuff stretching, and tucking</t>
+          <t>High — rolling, cuff stretching, and tucking</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — garment shape and tension must be inferred</t>
+          <t>Moderate — garment shape and tension must be inferred</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — material properties remain effectively constant</t>
+          <t>Low — material properties remain effectively constant</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — the socks can be unbundled without material alteration</t>
+          <t>Low — the socks can be unbundled without material alteration</t>
         </is>
       </c>
     </row>
@@ -1070,52 +1070,52 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
+          <t>Mixed manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed relative to the hand</t>
+          <t>Mixed relative to the hand</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — guided slider and constrained fabric deformation</t>
+          <t>Moderate — guided slider and constrained fabric deformation</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — alignment, tension, and guided motion</t>
+          <t>High — alignment, tension, and guided motion</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — engagement and disengagement</t>
+          <t>High — repeated engagement and disengagement of zipper teeth</t>
         </is>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — slider engagement and fabric tension must be detected</t>
+          <t>Moderate — slider engagement and fabric tension must be detected</t>
         </is>
       </c>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — material properties remain effectively constant</t>
+          <t>Low — material properties remain effectively constant</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — closing is reversed within the task</t>
+          <t>Low — closing is reversed within the task</t>
         </is>
       </c>
     </row>
@@ -1137,52 +1137,52 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deformable manipulanda / rigid environment</t>
+          <t>Deformable manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Larger than the hand</t>
+          <t>Larger than the hand</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — distributed sheet deformation</t>
+          <t>High — distributed sheet deformation</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — edge alignment and crease tolerance</t>
+          <t>Low — few environmental constraints on the sheet</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — support, folding, self-contact, and release</t>
+          <t>Low — few simple contact transitions during a single fold</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — alignment, deformation, and crease state must be monitored</t>
+          <t>Moderate — alignment, deformation, and crease state must be monitored</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — creasing changes local rest shape and stiffness</t>
+          <t>Moderate — creasing changes local rest shape and stiffness</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — unfolding leaves a persistent crease</t>
+          <t>Moderate — unfolding leaves a persistent crease</t>
         </is>
       </c>
     </row>
@@ -1204,52 +1204,52 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Direct</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
+          <t>Mixed manipulanda / rigid environment</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mixed relative to the hand</t>
+          <t>Mixed relative to the hand</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — seven objects and an elastic fastener</t>
+          <t>High — seven objects and an elastic fastener</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — alignment, compression, and wrapping</t>
+          <t>High — alignment, compression, and wrapping</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">High — gathering, stretching, and securing</t>
+          <t>High — gathering, stretching, and securing</t>
         </is>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Quasistatic</t>
+          <t>Quasistatic</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moderate — bundle geometry and band tension must be inferred</t>
+          <t>Moderate — bundle geometry and band tension must be inferred</t>
         </is>
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — material properties remain effectively constant</t>
+          <t>Low — material properties remain effectively constant</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Low — the bundle can be disassembled without material alteration</t>
+          <t>Low — the bundle can be disassembled without material alteration</t>
         </is>
       </c>
     </row>
@@ -1322,24 +1322,22 @@
           <t xml:space="preserve">Object Transport and Retrieval</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4</t>
-        </is>
+      <c r="C2" s="2">
+        <v>4</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25.0%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Pick Up Flat Object, Use Chopsticks, Blindly Retrieve an Object from Cover</t>
+          <t>Box and Blocks, Pick Up Flat Object, Use Chopsticks, Blindly Retrieve an Object from Cover</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5/5 categories (100.0%)</t>
+          <t>5/5 categories (100.0%)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1359,19 +1357,17 @@
           <t xml:space="preserve">Assembly and Fastening</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6</t>
-        </is>
+      <c r="C3" s="3">
+        <v>6</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">37.5%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peg-in-Hole, Twist Lid on Jar, Use Screwdriver, Fasten Button, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t>Peg-in-Hole, Twist Lid on Jar, Use Screwdriver, Fasten Button, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
@@ -1396,19 +1392,17 @@
           <t xml:space="preserve">Material Shaping and Reconfiguration</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4</t>
-        </is>
+      <c r="C4" s="2">
+        <v>4</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25.0%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie a Knot, In-Hand Reorienting, Bundle Socks, Paper Folding</t>
+          <t>Tie a Knot, In-Hand Reorienting, Bundle Socks, Paper Folding</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1433,19 +1427,17 @@
           <t xml:space="preserve">Opening, Separation, and Disassembly</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
+      <c r="C5" s="3">
+        <v>1</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Scissors</t>
+          <t>Use Scissors</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1470,19 +1462,17 @@
           <t xml:space="preserve">Dynamic Manipulation</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
+      <c r="C6" s="2">
+        <v>1</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spin a Top</t>
+          <t>Spin a Top</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1507,24 +1497,22 @@
           <t xml:space="preserve">Direct</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">13</t>
-        </is>
+      <c r="C7" s="3">
+        <v>13</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">81.3%</t>
+          <t>81.3%</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Fasten Button, In-Hand Reorienting, Spin a Top, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
+          <t>Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Fasten Button, In-Hand Reorienting, Spin a Top, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/2 categories (100.0%)</t>
+          <t>2/2 categories (100.0%)</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -1544,19 +1532,17 @@
           <t xml:space="preserve">Indirect</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
+      <c r="C8" s="2">
+        <v>3</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.8%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Screwdriver, Use Scissors, Use Chopsticks</t>
+          <t>Use Screwdriver, Use Scissors, Use Chopsticks</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1581,24 +1567,22 @@
           <t xml:space="preserve">Rigid manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">8</t>
-        </is>
+      <c r="C9" s="3">
+        <v>8</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">50.0%</t>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Twist Lid on Jar, Use Screwdriver, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover</t>
+          <t>Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Twist Lid on Jar, Use Screwdriver, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4/4 categories (100.0%)</t>
+          <t>4/4 categories (100.0%)</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1618,19 +1602,17 @@
           <t xml:space="preserve">Deformable manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
+      <c r="C10" s="2">
+        <v>3</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">18.8%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie a Knot, Bundle Socks, Paper Folding</t>
+          <t>Tie a Knot, Bundle Socks, Paper Folding</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -1655,19 +1637,17 @@
           <t xml:space="preserve">Mixed manipulanda / rigid environment</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4</t>
-        </is>
+      <c r="C11" s="3">
+        <v>4</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">25.0%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Scissors, Fasten Button, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t>Use Scissors, Fasten Button, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1692,19 +1672,17 @@
           <t xml:space="preserve">Rigid manipulandum / environment not engaged</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
+      <c r="C12" s="2">
+        <v>1</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">In-Hand Reorienting</t>
+          <t>In-Hand Reorienting</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1729,24 +1707,22 @@
           <t xml:space="preserve">Smaller than the hand</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4</t>
-        </is>
+      <c r="C13" s="3">
+        <v>4</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">25.0%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Pick Up Flat Object, Fasten Button, Spin a Top</t>
+          <t>Box and Blocks, Pick Up Flat Object, Fasten Button, Spin a Top</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">4/4 categories (100.0%)</t>
+          <t>4/4 categories (100.0%)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -1766,19 +1742,17 @@
           <t xml:space="preserve">Comparable to the hand</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5</t>
-        </is>
+      <c r="C14" s="2">
+        <v>5</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">31.3%</t>
+          <t>31.3%</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peg-in-Hole, Twist Lid on Jar, In-Hand Reorienting, Blindly Retrieve an Object from Cover, Bundle Socks</t>
+          <t>Peg-in-Hole, Twist Lid on Jar, In-Hand Reorienting, Blindly Retrieve an Object from Cover, Bundle Socks</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1803,19 +1777,17 @@
           <t xml:space="preserve">Larger than the hand</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
+      <c r="C15" s="3">
+        <v>1</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paper Folding</t>
+          <t>Paper Folding</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1840,19 +1812,17 @@
           <t xml:space="preserve">Mixed relative to the hand</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6</t>
-        </is>
+      <c r="C16" s="2">
+        <v>6</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">37.5%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie a Knot, Use Screwdriver, Use Scissors, Use Chopsticks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t>Tie a Knot, Use Screwdriver, Use Scissors, Use Chopsticks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1877,24 +1847,22 @@
           <t xml:space="preserve">Low</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5</t>
-        </is>
+      <c r="C17" s="3">
+        <v>6</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">31.3%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Twist Lid on Jar, Spin a Top</t>
+          <t>Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Twist Lid on Jar, In-Hand Reorienting, Spin a Top</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">3/3 categories (100.0%)</t>
+          <t>3/3 categories (100.0%)</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
@@ -1914,19 +1882,17 @@
           <t xml:space="preserve">Moderate</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4</t>
-        </is>
+      <c r="C18" s="2">
+        <v>4</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25.0%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Screwdriver, Fasten Button, Blindly Retrieve an Object from Cover, Zip a Zipper</t>
+          <t>Use Screwdriver, Fasten Button, Blindly Retrieve an Object from Cover, Zip a Zipper</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1951,19 +1917,17 @@
           <t xml:space="preserve">High</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7</t>
-        </is>
+      <c r="C19" s="3">
+        <v>6</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">43.8%</t>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie a Knot, Use Scissors, In-Hand Reorienting, Use Chopsticks, Bundle Socks, Paper Folding, Bundle Dowels with a Rubber Band</t>
+          <t>Tie a Knot, Use Scissors, Use Chopsticks, Bundle Socks, Paper Folding, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1988,24 +1952,22 @@
           <t xml:space="preserve">Low</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
-        </is>
+      <c r="C20" s="2">
+        <v>3</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12.5%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Spin a Top</t>
+          <t>Box and Blocks, Spin a Top, Paper Folding</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3/3 categories (100.0%)</t>
+          <t>3/3 categories (100.0%)</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -2025,19 +1987,17 @@
           <t xml:space="preserve">Moderate</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5</t>
-        </is>
+      <c r="C21" s="3">
+        <v>3</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">31.3%</t>
+          <t>18.8%</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Scissors, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Paper Folding</t>
+          <t>Use Scissors, Use Chopsticks, Blindly Retrieve an Object from Cover</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -2062,19 +2022,17 @@
           <t xml:space="preserve">High</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9</t>
-        </is>
+      <c r="C22" s="2">
+        <v>10</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">56.3%</t>
+          <t>62.5%</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t>Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -2099,29 +2057,27 @@
           <t xml:space="preserve">Low</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0</t>
-        </is>
+      <c r="C23" s="3">
+        <v>1</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t>Paper Folding</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/3 categories (66.7%)</t>
+          <t>3/3 categories (100.0%)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Coverage gap: no task has low constraint change.</t>
+          <t>Low, moderate, and high constraint change are represented; low is represented by only one task.</t>
         </is>
       </c>
     </row>
@@ -2136,19 +2092,17 @@
           <t xml:space="preserve">Moderate</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6</t>
-        </is>
+      <c r="C24" s="2">
+        <v>4</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">37.5%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Pick Up Flat Object, In-Hand Reorienting, Spin a Top, Use Chopsticks, Paper Folding</t>
+          <t>Box and Blocks, Pick Up Flat Object, Spin a Top, Use Chopsticks</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -2173,19 +2127,17 @@
           <t xml:space="preserve">High</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10</t>
-        </is>
+      <c r="C25" s="3">
+        <v>11</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">62.5%</t>
+          <t>68.8%</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Peg-in-Hole, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t>Peg-in-Hole, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -2210,24 +2162,22 @@
           <t xml:space="preserve">Quasistatic</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">15</t>
-        </is>
+      <c r="C26" s="2">
+        <v>15</v>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">93.8%</t>
+          <t>93.8%</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
+          <t>Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/2 categories (100.0%)</t>
+          <t>2/2 categories (100.0%)</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2247,19 +2197,17 @@
           <t xml:space="preserve">Dynamic</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
+      <c r="C27" s="3">
+        <v>1</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spin a Top</t>
+          <t>Spin a Top</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -2284,24 +2232,22 @@
           <t xml:space="preserve">Low</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4</t>
-        </is>
+      <c r="C28" s="2">
+        <v>4</v>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">25.0%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Spin a Top</t>
+          <t>Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Spin a Top</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3/3 categories (100.0%)</t>
+          <t>3/3 categories (100.0%)</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2321,19 +2267,17 @@
           <t xml:space="preserve">Moderate</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">11</t>
-        </is>
+      <c r="C29" s="3">
+        <v>11</v>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">68.8%</t>
+          <t>68.8%</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Use Chopsticks, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
+          <t>Tie a Knot, Twist Lid on Jar, Use Screwdriver, Use Scissors, Fasten Button, In-Hand Reorienting, Use Chopsticks, Bundle Socks, Zip a Zipper, Paper Folding, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -2358,19 +2302,17 @@
           <t xml:space="preserve">High</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
+      <c r="C30" s="2">
+        <v>1</v>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Blindly Retrieve an Object from Cover</t>
+          <t>Blindly Retrieve an Object from Cover</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -2395,24 +2337,22 @@
           <t xml:space="preserve">Low</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14</t>
-        </is>
+      <c r="C31" s="3">
+        <v>14</v>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">87.5%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t>Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2/3 categories (66.7%)</t>
+          <t>2/3 categories (66.7%)</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -2432,19 +2372,17 @@
           <t xml:space="preserve">Moderate</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
-        </is>
+      <c r="C32" s="2">
+        <v>2</v>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">12.5%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Scissors, Paper Folding</t>
+          <t>Use Scissors, Paper Folding</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -2469,19 +2407,17 @@
           <t xml:space="preserve">High</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0</t>
-        </is>
+      <c r="C33" s="3">
+        <v>0</v>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.0%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t/>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -2506,24 +2442,22 @@
           <t xml:space="preserve">Low</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14</t>
-        </is>
+      <c r="C34" s="2">
+        <v>14</v>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">87.5%</t>
+          <t>87.5%</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
+          <t>Box and Blocks, Peg-in-Hole, Pick Up Flat Object, Tie a Knot, Twist Lid on Jar, Use Screwdriver, Fasten Button, In-Hand Reorienting, Spin a Top, Use Chopsticks, Blindly Retrieve an Object from Cover, Bundle Socks, Zip a Zipper, Bundle Dowels with a Rubber Band</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3/3 categories (100.0%)</t>
+          <t>3/3 categories (100.0%)</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -2543,19 +2477,17 @@
           <t xml:space="preserve">Moderate</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
+      <c r="C35" s="3">
+        <v>1</v>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paper Folding</t>
+          <t>Paper Folding</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -2580,19 +2512,17 @@
           <t xml:space="preserve">High</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
+      <c r="C36" s="2">
+        <v>1</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.3%</t>
+          <t>6.3%</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Use Scissors</t>
+          <t>Use Scissors</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -2653,7 +2583,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The hand acts directly on the task object.</t>
+          <t>The hand acts directly on the task object.</t>
         </is>
       </c>
     </row>
@@ -2670,7 +2600,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tools transmit the hand’s action to the task object.</t>
+          <t>Tools transmit the hand’s action to the task object.</t>
         </is>
       </c>
     </row>
@@ -2687,7 +2617,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid objects and tools interact with rigid supports or fixtures.</t>
+          <t>Rigid objects and tools interact with rigid supports or fixtures.</t>
         </is>
       </c>
     </row>
@@ -2704,7 +2634,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Deformable objects are handled using rigid supports or fixtures.</t>
+          <t>Deformable objects are handled using rigid supports or fixtures.</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2651,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rigid and deformable components are handled together in a rigid environment.</t>
+          <t>Rigid and deformable components are handled together in a rigid environment.</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2668,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">A rigid object is manipulated within the hand without environmental contact.</t>
+          <t>A rigid object is manipulated within the hand without environmental contact.</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2685,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The main handled object or component is smaller than the hand.</t>
+          <t>The main handled object or component is smaller than the hand.</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2702,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">The handled object is approximately the size of the hand.</t>
+          <t>The handled object is approximately the size of the hand.</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2719,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The handled object extends beyond the hand’s size.</t>
+          <t>The handled object extends beyond the hand’s size.</t>
         </is>
       </c>
     </row>
@@ -2806,7 +2736,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handled components or relevant dimensions span multiple size categories.</t>
+          <t>Handled components or relevant dimensions span multiple size categories.</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2753,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">One rigid object is controlled with a simple grasp and minimal contact reconfiguration.</t>
+          <t>One rigid object is controlled at a time.</t>
         </is>
       </c>
     </row>
@@ -2840,7 +2770,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Guided mechanisms, localized deformation, or movable distractors require limited additional coordination.</t>
+          <t>Guided mechanisms, localized deformation, or movable distractors require limited additional coordination.</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2787,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiple objects, distributed deformation, or independent finger-contact motion require substantial coordination.</t>
+          <t>Multiple independently controlled components or distributed deformation require substantial coordination.</t>
         </is>
       </c>
     </row>
@@ -2874,7 +2804,7 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Few simultaneous constraints leave broad freedom in grasp and motion.</t>
+          <t>Few simultaneous constraints leave broad freedom in grasp and motion.</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2821,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Alignment, confinement, or contact-force requirements allow several feasible manipulation strategies.</t>
+          <t>Alignment, confinement, or contact-force requirements allow several feasible manipulation strategies.</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2838,7 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tight geometry, restricted access, topology, or coupled force requirements severely limit feasible grasps and motions.</t>
+          <t>Restrictive geometry, topology, or coupled contact modes and forces strongly constrain manipulation.</t>
         </is>
       </c>
     </row>
@@ -2925,7 +2855,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contacts and motion restrictions remain effectively constant.</t>
+          <t>Few simple contact transitions introduce limited motion restrictions.</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2872,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contacts follow a limited sequence, shift within a grasp, or repeat the same handling cycle.</t>
+          <t>Support transfers or repeated handling cycles change contact constraints in a predictable sequence.</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2889,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Contact modes progressively restrict motion or repeatedly reorganize across interfaces or deformable objects.</t>
+          <t>Contact modes reorganize, mating interfaces engage or disengage, or deformable self-contacts evolve.</t>
         </is>
       </c>
     </row>
@@ -2976,7 +2906,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Controlled positioning and contact forces suffice; exploiting momentum is unnecessary.</t>
+          <t>Controlled positioning and contact forces suffice; exploiting momentum is unnecessary.</t>
         </is>
       </c>
     </row>
@@ -2993,7 +2923,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Success requires deliberately generating or exploiting momentum and inertial effects.</t>
+          <t>Success requires deliberately generating or exploiting momentum and inertial effects.</t>
         </is>
       </c>
     </row>

</xml_diff>